<commit_message>
Actualización automática de noticias
</commit_message>
<xml_diff>
--- a/Data/Lambayeque/noticias_lambayeque_20260904_20260911.xlsx
+++ b/Data/Lambayeque/noticias_lambayeque_20260904_20260911.xlsx
@@ -470,10 +470,53 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Conoce las 125 agencias donde el Reniec brindará atención especial este fin de semana</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>La atención del sábado se realizará en agencias de Piura, La Libertad, Lambayeque, Tumbes, Cajamarca, San Martín, Loreto, Áncash, Junín, Ayacucho, Arequipa, Cusco, Lima, Puno, Ica, Ucayali, Huancavelica, Madre de Dios y Amazonas.
+En tanto, el domingo, el Reniec continuará atendiendo en Piura, Lambayeque, Tumbes, Lima y Puno, de 8:15 a.
+m.
+a 12:45 p.
+m.
+Conoce aquí las agencias, centros de atención y horarios habilitados para este fin de semana: Enlace: https://docs.google.com/spreadsheets/d/1TnRZB_IOqx5TS8fzKlCfA2gmvg2oovzQ/edit?gid=154156413#gid=154156413 Lima Metropolitana y Callao: atención este sábado En Lima Metropolitana y Callao, el Reniec atenderá este sábado 12 de setiembre en seis centros, donde los ciudadanos podrán realizar trámites y recoger sus documentos de identidad.
+La atención será de 8:15 a.
+m.
+a 12:45 p.
+m.
+en MAC Callao, MAC Lima Este, MAC Lima Norte, MAC Lima Sur, MAC Ventanilla y la agencia de Miraflores.
+Esta atención especial busca ampliar las opciones para quienes, por sus actividades durante la semana, requieren realizar sus trámites o recoger su DNI durante el fin de semana, especialmente ante la proximidad de las Elecciones Regionales y Municipales (ERM) 2026.
+Atención el domingo 13 en cinco regiones El domingo 13 de setiembre, el Reniec continuará atendiendo en 13 centros ubicados en Piura, Lambayeque, Tumbes, Lima y Puno, de 8:15 a.
+m.
+a 12:45 p.
+m.
+En Lima, funcionarán los centros de atención de Independencia y Cercado de Lima, en el mismo horario.
+Conoce aquí las agencias, centros de atención y horarios habilitados para este fin de semana: Enlace: https://docs.google.com/spreadsheets/d/1TnRZB_IOqx5TS8fzKlCfA2gmvg2oovzQ/edit?gid=154156413#gid=154156413 Lea también: Reniec tomará gratis la foto para DNI de niños: conoce en qué sedes y cómo hacerlo ¿Dónde consultar si mi DNI se encuentra listo para recogerlo? Los ciudadanos deben acceder a la página oficial de Reniec a través de este Enlace: https://serviciosportal.reniec.gob.pe/cetdnipi/inicio.htm ingresar su número de DNI o de solicitud, hacer clic en ‘Consultar’ y, de inmediato, les aparecerá sus datos completos, la sede que eligieron para el recojo de su DNI y si el estado de su trámite se encuentra al 100%, listo para recoger su documento.
+Más en Andina: La Autoridad Nacional de Infraestructura (ANIN) amplió su cartera de intervención integral para el control de riesgos por movimientos de masa e inundaciones en la cuenca del río Rímac con la incorporación de las quebradas Vizcachera, Ñaña y La Laguna ?? https://t.co/T25qFB3xn7 pic.twitter.com/vrqvZ2YCgN — Agencia Andina (@Agencia_Andina) September 10, 2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-conoce-las-125-agencias-donde-reniec-brindara-atencion-especial-este-fin-semana-1091330.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Papa León XIV: visitan pampas de Pimentel, escenario previsto para multitudinaria misa</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Como parte de estos trabajos, representantes de las instituciones involucradas participaron este jueves en una reunión de coordinación que incluyó una visita de reconocimiento a las pampas de Pimentel, escenario previsto para las actividades multitudinarias.
 La jornada se desarrolló en dos etapas.
@@ -488,27 +531,27 @@
 ?? https://t.co/QxyDxlNq8H pic.twitter.com/3a2X15pY1D — Agencia Andina (@Agencia_Andina) September 11, 2026</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>https://andina.pe/agencia/noticia-papa-leon-xiv-visitan-pampas-pimentel-escenario-previsto-para-multitudinaria-misa-1091314.aspx</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Andina</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B4" s="2" t="n">
         <v>46275</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Productores de Piura mejorarán producción de forraje caprino con ayuda tecnológica de INIA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>La actividad, desarrollada a través de la Estación Experimental Agraria El Chira (EEA Chira), como parte de las acciones del Proyecto Caprinos Procap, está dirigida a productores de la Asociación Agraria Alfa y Omega, con el propósito de fortalecer el manejo integral del sistema productivo, promoviendo una adecuada relación entre la conservación de la fertilidad del suelo, el establecimiento de especies forrajeras y la disponibilidad de alimento de calidad para los animales.
 Durante el desarrollo de las jornadas técnicas, especialistas del INIA capacitaron a los productores en la selección y el uso de semillas de alta calidad, evaluación de la fertilidad del suelo, preparación del terreno, elaboración de planes de fertilización, establecimiento y manejo de pastos mejorados, producción y aplicación de abonos orgánicos, así como en prácticas orientadas a conservar la capacidad productiva del suelo.
@@ -522,27 +565,27 @@
 La Geresa reforzó las acciones de prevención y control, especialmente en Chiclayo, La Victoria y Motupe.?? https://t.co/MjncOyjiFL pic.twitter.com/l13jzOYyy5 — Agencia Andina (@Agencia_Andina) September 10, 2026</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>https://andina.pe/agencia/noticia-productores-piura-mejoraran-produccion-forraje-caprino-ayuda-tecnologica-inia-1091279.aspx</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Andina</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B5" s="2" t="n">
         <v>46275</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Región Lambayeque reporta 13 defunciones y cerca de 4,000 afectados a causa del dengue</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>El gerente regional de Salud, Yonny Ureta Núñez , explicó que durante las visitas domiciliarias realizadas por las brigadas sanitarias se viene detectando de manera recurrente la presencia de larvas en floreros que contienen agua , especialmente en las principales ciudades de la región, entre ellas Chiclayo.
 Ante esta situación, recomendó a las familias reemplazar el agua de los floreros por arena húmeda, además de eliminar o mantener adecuadamente tapados todos los recipientes que puedan acumular agua y convertirse en criaderos del mosquito Aedes aegypti.
@@ -562,27 +605,27 @@
 ?? https://t.co/zTE0Rrb3mx pic.twitter.com/uQKWkNBvVY — Agencia Andina (@Agencia_Andina) September 10, 2026</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://andina.pe/agencia/noticia-region-lambayeque-reporta-13-defunciones-y-cerca-4000-afectados-a-causa-del-dengue-1091276.aspx</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Andina</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>46275</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Tragedia vial en Pasco: despiste de vehículo en la vía a Oxapampa deja siete fallecidos</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Se informó que el accidente habría sido provocado por un despiste que sufrió la unidad, identificada con la placa W4S.444, perteneciente a la empresa Virgen del Carmen.
 Tras conocerse la tragedia vial , hasta el lugar llegaron efectivos de la Policía Nacional y serenos del distrito de Ninacaca, quienes acordonaron la zona y realizaron las primeras diligencias para verificar la magnitud del siniestro.
@@ -599,47 +642,9 @@
 ?? https://t.co/ARvk5P1G8l pic.twitter.com/pYb4tiStO4 — Agencia Andina (@Agencia_Andina) September 10, 2026</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://andina.pe/agencia/noticia-tragedia-vial-pasco-despiste-vehiculo-la-via-a-oxapampa-deja-siete-fallecidos-1091269.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Andina</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>León XIV pone a Lambayeque en los ojos del mundo y busca dar salto de desarrollo turístico</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>El diagnóstico, elaborado con revisión documental, entrevistas y mesas técnicas en Chiclayo, Ferreñafe y Lambayeque, recogió la opinión de más de 85 actores públicos, privados y académicos.
-El estudio que fue presentado oficialmente en esta ciudad identificó 204 recursos turísticos inventariados y destacó que el Santuario Histórico Bosque de Pómac posee jerarquía 4, el mismo nivel asignado a Machu Picchu.
-La Decana del Colegio Profesional de Licenciados en Turismo de Lambayeque y responsable de este estudio, Rosse Marie Esparza Huamanchumo, informó a la Agencia Andina que uno de los principales desafíos está en elevar la calidad de los servicios.
-“Hasta abril de 2026 se registraban 751 establecimientos de hospedaje, mientras que solo 54 restaurantes figuraban calificados y categorizados por la autoridad turística regional.
-En Ferreñafe, además, no había ningún restaurante categorizado”, alertó.
-El plan advierte que Lambayeque no podrá consolidarse como destino competitivo si no enfrenta problemas como la informalidad, deficiente limpieza, seguridad, limitada infraestructura turística y falta de articulación entre autoridades, empresarios y otros actores del sector.
-Indicó que la propuesta plantea fortalecer la gobernanza, mejorar la infraestructura y seguridad turística, formalizar y capacitar a los prestadores de servicios e impulsar la transformación digital, especialmente para conectar con las nuevas generaciones de viajeros.
-“La coyuntura del Papa León XIV y su histórica vinculación pastoral con Lambayeque es considerada una oportunidad excepcional para reposicionar la región.
-Entre los atractivos que se plantea potenciar figuran Ciudad Eten, reconocida como ciudad eucarística, la Cruz de Motupe y el Divino Niño del Milagro, además de los espacios vinculados a la denominada Ruta del Papa León XIV”, apuntó.
-Mencionó, además, que la estrategia también contempla aprovechar la futura construcción del terminal marítimo multipropósito de Puerto Eten, prevista en el horizonte de 2030, y modernizar el aeropuerto internacional José Abelardo Quiñones para incrementar la conectividad aérea y atraer nuevos vuelos.
-Refirió igualmente, que entre las metas destacan la elaboración de 12 planes de desarrollo turístico local, la creación de seis circuitos turísticos temáticos y la implementación de un Observatorio Turístico Regional que permita contar con información precisa sobre visitantes, consumo y comportamiento de la actividad turística.
-Subrayó que el gran reto será que el plan no quede como un documento más.
-“Su ejecución requiere el compromiso conjunto del Gobierno Regional, municipalidades, empresarios, academia y organizaciones vinculadas al turismo, con acciones concretas que permitan convertir la riqueza de Lambayeque en desarrollo económico sostenible”, apuntó.
-Más en Andina:</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://andina.pe/agencia/noticia-leon-xiv-pone-a-lambayeque-los-ojos-del-mundo-y-busca-dar-salto-desarrollo-turistico-1091264.aspx</t>
         </is>
       </c>
     </row>

</xml_diff>